<commit_message>
Correct G2 chapter image page bindings and log text-only B comparison
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/authoring/g2-completion/G2-CH1-ARENA-IMAGE-PASS-A-PARTIAL-v0.1.xlsx
+++ b/authoring/g2-completion/G2-CH1-ARENA-IMAGE-PASS-A-PARTIAL-v0.1.xlsx
@@ -1412,7 +1412,7 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 010؛ SHA تصویر c3474a5e6f98؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 007؛ SHA تصویر 83670103837e؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>بالا: عنوان فصل و پلاک؛ میانه: عکس گله؛ پایین: متن گفت‌وگو. شمارهٔ چاپی در پاصفحه آشکار نیست؛ صفحهٔ ۱ از عنوان/ترتیب استنباط شده. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>بالا: عنوان فصل و پلاک؛ میانه: عکس گله؛ پایین: متن گفت‌وگو. شمارهٔ چاپی در پاصفحه آشکار نیست؛ صفحهٔ ۱ از عنوان/ترتیب استنباط شده. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 003؛ SHA تصویر 7c71178eb960؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 008؛ SHA تصویر fa215bd290de؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>بالا: سؤال شمارش به توپ‌ها اشاره دارد؛ پایین: دستور «هر کدام چه عددی» به شکل‌های جدا و جای‌خالی زیر هر شکل مربوط است. پاصفحه ۲ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>بالا: سؤال شمارش به توپ‌ها اشاره دارد؛ پایین: دستور «هر کدام چه عددی» به شکل‌های جدا و جای‌خالی زیر هر شکل مربوط است. پاصفحه ۲ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 007؛ SHA تصویر 83670103837e؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 009؛ SHA تصویر b65ca6559534؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>دستور بالای صفحه به گونه‌های گل در باغچه و ردیف‌های جدول میانی وصل است؛ جدول پایین فعالیت دیگری است. شمار جزءِ هر نوع هنوز دوباره‌شماری مستقل نشده؛ پاصفحه ۳ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>دستور بالای صفحه به گونه‌های گل در باغچه و ردیف‌های جدول میانی وصل است؛ جدول پایین فعالیت دیگری است. شمار جزءِ هر نوع هنوز دوباره‌شماری مستقل نشده؛ پاصفحه ۳ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 009؛ SHA تصویر b65ca6559534؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 010؛ SHA تصویر c3474a5e6f98؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>شماره‌های تمرین ۱ تا ۳ به سه ناحیهٔ جدا مربوط‌اند؛ مقایسهٔ گل‌ها در قاب پایین «حدس بزن» است. پاصفحه ۴ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>شماره‌های تمرین ۱ تا ۳ به سه ناحیهٔ جدا مربوط‌اند؛ مقایسهٔ گل‌ها در قاب پایین «حدس بزن» است. پاصفحه ۴ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>هر جدول دهگان/یکی کنار همان آرایش میله‌هاست؛ کارت‌های پایین تمرین ساخت عدد است. پاصفحه ۵ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>هر جدول دهگان/یکی کنار همان آرایش میله‌هاست؛ کارت‌های پایین تمرین ساخت عدد است. پاصفحه ۵ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 016؛ SHA تصویر 77e476760837؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 012؛ SHA تصویر d8651762e519؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>سؤال بالا به گل‌های همان ناحیه پیوند دارد؛ پایین برچسب دهگان/یکان به جدول مجاور مربوط است. شمار گل هنوز دوباره‌شماری مستقل نشده؛ پاصفحه ۶ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>سؤال بالا به گل‌های همان ناحیه پیوند دارد؛ پایین برچسب دهگان/یکان به جدول مجاور مربوط است. شمار گل هنوز دوباره‌شماری مستقل نشده؛ پاصفحه ۶ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>هر جای‌خالی فقط به توالی یا جدول همان بخش تعلق دارد؛ قاب الگویابی پایین فعالیت دیگری است. پاصفحه ۷ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>هر جای‌خالی فقط به توالی یا جدول همان بخش تعلق دارد؛ قاب الگویابی پایین فعالیت دیگری است. پاصفحه ۷ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>میله‌های سبز به مسئلهٔ کتاب‌ها وصل‌اند؛ مثلث‌ها برای خواندن عدد و «پنجمین بعد» هستند؛ دو قاب جانور برای مقایسهٔ بیش از ۲۰ است. شمارش تک‌به‌تک شکل‌ها نیازمند بازبین دوم؛ پاصفحه ۸ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>میله‌های سبز به مسئلهٔ کتاب‌ها وصل‌اند؛ مثلث‌ها برای خواندن عدد و «پنجمین بعد» هستند؛ دو قاب جانور برای مقایسهٔ بیش از ۲۰ است. شمارش تک‌به‌تک شکل‌ها نیازمند بازبین دوم؛ پاصفحه ۸ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>نقشهٔ پایین یک شکل نیمه‌کامل است، نه شکل آمادهٔ پاسخ؛ جهت خطوط و جای قطعهٔ رنگی برای دستور تکمیل مهم‌اند. پاصفحه ۹ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>نقشهٔ پایین یک شکل نیمه‌کامل است، نه شکل آمادهٔ پاسخ؛ جهت خطوط و جای قطعهٔ رنگی برای دستور تکمیل مهم‌اند. پاصفحه ۹ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 012؛ SHA تصویر d8651762e519؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 016؛ SHA تصویر 77e476760837؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>هر محور به عبارت بلافاصله کنار آن مربوط است؛ خانه‌های رنگی به دستور جمع همان ردیف مربوط‌اند. پاصفحه ۱۰ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>هر محور به عبارت بلافاصله کنار آن مربوط است؛ خانه‌های رنگی به دستور جمع همان ردیف مربوط‌اند. پاصفحه ۱۰ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>عکس مهره‌ها به فعالیت دو نفره مربوط است؛ ساعت‌های پایین بخش جداگانه‌اند و از عبارت‌های جمع میانه پاسخ‌گیری نمی‌کنند. پاصفحه ۱۱ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>عکس مهره‌ها به فعالیت دو نفره مربوط است؛ ساعت‌های پایین بخش جداگانه‌اند و از عبارت‌های جمع میانه پاسخ‌گیری نمی‌کنند. پاصفحه ۱۱ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>تصویر خصوصی 008؛ SHA تصویر fa215bd290de؛ PDF C205 تطبیق بایتی نشده</t>
+          <t>تصویر خصوصی 018؛ SHA تصویر 0f0f5bcf7673؛ PDF C205 تطبیق بایتی نشده</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>محورها با عبارت‌های جمع/تفریقِ کنار همان ردیف پیوند دارند؛ طرح مثلثیِ پایین نمونهٔ کاردستی است، نه پاسخ عددی عبارت‌ها. پاصفحه ۱۲ دیده شد. خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
+          <t>محورها با عبارت‌های جمع/تفریقِ کنار همان ردیف پیوند دارند؛ طرح مثلثیِ پایین نمونهٔ کاردستی است، نه پاسخ عددی عبارت‌ها. پاصفحه ۱۲ دیده شد. نگاشت PNG↔صفحه پس از خطای نسخهٔ اولیه اصلاح شد؛ خوانش A محدود؛ نه مهر/نه OCR؛ منشأ بایت PDF نامعلوم.</t>
         </is>
       </c>
     </row>

</xml_diff>